<commit_message>
Update inventory via Streamlit
</commit_message>
<xml_diff>
--- a/Inventory.xlsx
+++ b/Inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H165"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5858,6 +5858,36 @@
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr"/>
     </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Pendrive 32 GB</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>4</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>G1-Office-Stationary Storage</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>